<commit_message>
Update data 28/06: sembako, sentimen, pakan, peternakan + precompute fix
</commit_message>
<xml_diff>
--- a/data/harga_pakan_ternak.xlsx
+++ b/data/harga_pakan_ternak.xlsx
@@ -81,7 +81,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -95,11 +95,14 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -129,6 +132,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -496,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y61"/>
+  <dimension ref="A1:Y62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5557,6 +5566,85 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B62" s="12" t="n">
+        <v>4896</v>
+      </c>
+      <c r="C62" s="12" t="n">
+        <v>7984</v>
+      </c>
+      <c r="D62" s="12" t="n">
+        <v>4039</v>
+      </c>
+      <c r="E62" s="12" t="n">
+        <v>8023</v>
+      </c>
+      <c r="F62" s="12" t="n">
+        <v>4764</v>
+      </c>
+      <c r="G62" s="12" t="n">
+        <v>4168</v>
+      </c>
+      <c r="H62" s="12" t="n">
+        <v>8149</v>
+      </c>
+      <c r="I62" s="12" t="n">
+        <v>7908</v>
+      </c>
+      <c r="J62" s="12" t="n">
+        <v>3637</v>
+      </c>
+      <c r="K62" s="12" t="n">
+        <v>8637</v>
+      </c>
+      <c r="L62" s="12" t="n">
+        <v>3202</v>
+      </c>
+      <c r="M62" s="12" t="n">
+        <v>8201</v>
+      </c>
+      <c r="N62" s="12" t="n">
+        <v>3582</v>
+      </c>
+      <c r="O62" s="12" t="n">
+        <v>8038</v>
+      </c>
+      <c r="P62" s="12" t="n">
+        <v>2830</v>
+      </c>
+      <c r="Q62" s="12" t="n">
+        <v>2386</v>
+      </c>
+      <c r="R62" s="12" t="n">
+        <v>8059</v>
+      </c>
+      <c r="S62" s="12" t="n">
+        <v>4006</v>
+      </c>
+      <c r="T62" s="12" t="n">
+        <v>5148</v>
+      </c>
+      <c r="U62" s="12" t="n">
+        <v>5211</v>
+      </c>
+      <c r="V62" s="12" t="n">
+        <v>7515</v>
+      </c>
+      <c r="W62" s="12" t="n">
+        <v>4933</v>
+      </c>
+      <c r="X62" s="12" t="n">
+        <v>3332</v>
+      </c>
+      <c r="Y62" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>